<commit_message>
가람: Decision & AI Usage Log xlsx에 발표자료 재구성 행 추가
md 로그(decision-log, ai-usage-log)에 기록한 08.21 항목을
제출용 03_Decision_AI_Usage_Log.xlsx의 A4·B5 전수 시트에도 동기화.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/진정가_CardFit_역기획프로젝트_Final/03_Decision_AI_Usage_Log.xlsx
+++ b/진정가_CardFit_역기획프로젝트_Final/03_Decision_AI_Usage_Log.xlsx
@@ -956,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2152,6 +2152,48 @@
       <c r="H31" s="5" t="inlineStr">
         <is>
           <t>조건부 반영(폴더·추적표는 반영, 문제정의 문구는 07 JTBD 확정 전 🟠 미승인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>김가람</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>발표자료 10분 재구성(18슬라이드) + 2부 구성 발표대본 작성</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Claude로 "PPT 발표용 재구성 및 디자인 수정 프롬프트"를 실행 — 기존 발표자료의 내용·문구·수치는 임의 변경 금지, 순서·분량·레이아웃·정렬·디자인만 개선하도록 범위 한정. 슬라이드 구성에 맞춰 0:00~5:00(슬라이드 1~9)·5:00~10:00(슬라이드 10~18) 2부 발표대본을 별도 작성</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>결과물 대조 검증 결과 핵심 수치·사실(1,473만~2,203만원, 88.4%, F-04, 40%, Concierge Test 등)이 그대로 보존됨. Cover 페이지 요구사항(서비스명 CardFit 대문자 표기, 태그라인 "과거 분석을 넘어, 미래 지출을 설계하다", 팀명 진정가·팀원 jennie/annie/cindy, 지정 문구 삭제)이 지시대로 정확히 반영됨</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>이 행은 완성된 프롬프트·결과 파일만 대조해 작성됨 — 실제 작업 세션 중 반복 수정 과정은 확인할 수 없어 비워둠. 실제 브라우저 렌더링에서 여백·정렬이 지시대로 개선됐는지도 육안 검증이 필요함</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>(가람 본인 확인·보완 필요 — 이 행은 결과물 대조만으로 작성됨)</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>조건부 반영(수치·사실 보존은 확인, 디자인 품질은 육안 검증 대기)</t>
         </is>
       </c>
     </row>
@@ -3087,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3114,7 +3156,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8950,6 +8991,48 @@
       <c r="H142" s="5" t="inlineStr">
         <is>
           <t>외부 CDN(Tailwind·Pretendard)에 의존해 오프라인에서는 스타일이 깨질 수 있음 — 발표 환경에 인터넷 연결 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21 (금)</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>가람</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>최종 발표자료 분량 — 🔹 기존 30슬라이드(15분 대본 기준) 유지 🔹 10분 발표용 18슬라이드로 재구성</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>실제 발표 시간이 10분으로 제약되어 있어, 기존 30슬라이드/15분 대본 구성으로는 시간을 맞출 수 없음. "PPT 발표용 재구성 및 디자인 수정 프롬프트"로 범위를 내용·수치 변경 없이 순서·통합·디자인 개선으로만 한정</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>② — 발표 시나리오 순서에 맞춰 18슬라이드로 통합·축소(CardFit_Deck_10min_v2-2.html), 0:00~5:00(슬라이드 1~9)·5:00~10:00(슬라이드 10~18) 2부 발표대본 신규 작성(CardFit_발표대본.pdf). Cover 문구·팀정보(서비스명 CardFit, 태그라인 "과거 분석을 넘어, 미래 지출을 설계하다", 팀명 진정가·팀원 jennie/annie/cindy) 확정</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>기존 자료가 15분 발표 기준으로 작성돼 10분 제약과 맞지 않음</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>실제 리허설 결과 10분을 초과하거나 미달하면 슬라이드 수·대본 재조정</t>
         </is>
       </c>
     </row>

</xml_diff>